<commit_message>
Frontend + backend đồng bộ, form nhập tay + báo giá AI
</commit_message>
<xml_diff>
--- a/pricing.xlsx
+++ b/pricing.xlsx
@@ -451,7 +451,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -802,9 +802,103 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>DH1774582247169</v>
+      </c>
+      <c r="B9" t="str">
+        <v>3/27/2026, 10:30:47 AM</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Chiến</v>
+      </c>
+      <c r="D9" t="str">
+        <v>0916426966</v>
+      </c>
+      <c r="E9" t="str">
+        <v>hop-gai-001</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Hộp gài</v>
+      </c>
+      <c r="G9">
+        <v>2000</v>
+      </c>
+      <c r="H9">
+        <v>700</v>
+      </c>
+      <c r="I9">
+        <v>400</v>
+      </c>
+      <c r="J9">
+        <v>800000</v>
+      </c>
+      <c r="K9">
+        <v>1400000</v>
+      </c>
+      <c r="L9">
+        <v>600000</v>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v>bao_gia</v>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>DH1774583534259</v>
+      </c>
+      <c r="B10" t="str">
+        <v>3/27/2026, 10:52:14 AM</v>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v>hop-gai-001</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Hộp gài</v>
+      </c>
+      <c r="G10">
+        <v>100</v>
+      </c>
+      <c r="H10">
+        <v>700</v>
+      </c>
+      <c r="I10">
+        <v>400</v>
+      </c>
+      <c r="J10">
+        <v>40000</v>
+      </c>
+      <c r="K10">
+        <v>70000</v>
+      </c>
+      <c r="L10">
+        <v>30000</v>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v>bao_gia</v>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O10"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>